<commit_message>
12 W Palmer: owner died 9/2/2025 after judgment; gut + foundation scenarios, max bid cut to $135k
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VbrkCepGz7t37qyR3xqDEz
</commit_message>
<xml_diff>
--- a/deep-dives/12-w-palmer/12_w_palmer_scenarios.xlsx
+++ b/deep-dives/12-w-palmer/12_w_palmer_scenarios.xlsx
@@ -485,7 +485,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="247">
   <si>
     <t xml:space="preserve">Sheriff Sale Underwriting Model, Philadelphia Nov 3 2026</t>
   </si>
@@ -992,6 +992,30 @@
   </si>
   <si>
     <t xml:space="preserve">2nd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1311511-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 Gut + $30k foundation, ARV 675k, vacant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1311511-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Gut + $30k foundation, ARV 640k, vacant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1311511-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 Gut + $30k foundation, ARV 710k, vacant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1311511-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 Gut + $30k foundation, ARV 675k, + $15k estate/title cure</t>
   </si>
   <si>
     <t xml:space="preserve">Property</t>
@@ -3001,108 +3025,260 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="8"/>
+      <c r="A9" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>19125</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>27200</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>329601</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>1728</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>1113</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>1925</v>
+      </c>
+      <c r="J9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>409100</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>330000</v>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>675000</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>3200</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="Q9" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="R9" s="8" t="n">
+        <v>2500</v>
+      </c>
       <c r="S9" s="8"/>
       <c r="T9" s="8"/>
       <c r="U9" s="16"/>
       <c r="V9" s="19"/>
       <c r="W9" s="8"/>
-      <c r="X9" s="11"/>
+      <c r="X9" s="11" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="8"/>
+      <c r="A10" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>19125</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>27200</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>329601</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>1728</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>1113</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>1925</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>409100</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>330000</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>640000</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>3200</v>
+      </c>
+      <c r="O10" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="R10" s="8" t="n">
+        <v>2500</v>
+      </c>
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
       <c r="U10" s="16"/>
       <c r="V10" s="19"/>
       <c r="W10" s="8"/>
-      <c r="X10" s="11"/>
+      <c r="X10" s="11" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="8"/>
+      <c r="A11" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>19125</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>27200</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>329601</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>1728</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>1113</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>1925</v>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>409100</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>330000</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>710000</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>3200</v>
+      </c>
+      <c r="O11" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="P11" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="Q11" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="R11" s="8" t="n">
+        <v>2500</v>
+      </c>
       <c r="S11" s="8"/>
       <c r="T11" s="8"/>
       <c r="U11" s="16"/>
       <c r="V11" s="19"/>
       <c r="W11" s="8"/>
-      <c r="X11" s="11"/>
+      <c r="X11" s="11" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="8"/>
+      <c r="A12" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>19125</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>27200</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>329601</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>1728</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>1113</v>
+      </c>
+      <c r="I12" s="16" t="n">
+        <v>1925</v>
+      </c>
+      <c r="J12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>409100</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>330000</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>675000</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>3200</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>17500</v>
+      </c>
       <c r="S12" s="8"/>
       <c r="T12" s="8"/>
       <c r="U12" s="16"/>
       <c r="V12" s="19"/>
       <c r="W12" s="8"/>
-      <c r="X12" s="11"/>
+      <c r="X12" s="11" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
@@ -3932,11 +4108,11 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="20" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="D1" s="21"/>
       <c r="E1" s="21"/>
@@ -3946,18 +4122,18 @@
       <c r="I1" s="21"/>
       <c r="J1" s="21"/>
       <c r="K1" s="6" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
       <c r="N1" s="7"/>
       <c r="O1" s="6" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="S1" s="7"/>
       <c r="T1" s="7"/>
@@ -3967,7 +4143,7 @@
       <c r="X1" s="7"/>
       <c r="Y1" s="7"/>
       <c r="Z1" s="6" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="AA1" s="7"/>
       <c r="AB1" s="7"/>
@@ -3980,10 +4156,10 @@
       <c r="AI1" s="7"/>
       <c r="AJ1" s="7"/>
       <c r="AK1" s="6" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="AL1" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="AM1" s="7"/>
       <c r="AN1" s="7"/>
@@ -3996,118 +4172,118 @@
         <v>129</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="AB2" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="AE2" s="5" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="AG2" s="5" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="AH2" s="5" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="AI2" s="5" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="AJ2" s="5" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="AK2" s="5" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="AL2" s="5" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="AM2" s="5" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="AN2" s="5" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5082,154 +5258,154 @@
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="str">
         <f aca="false">IF(Deals!A9="","",Deals!A9)</f>
-        <v/>
+        <v>1311511-6</v>
       </c>
       <c r="B9" s="0" t="str">
         <f aca="false">IF(A9="","",Deals!B9)</f>
-        <v/>
+        <v>6 Gut + $30k foundation, ARV 675k, vacant</v>
       </c>
       <c r="C9" s="21" t="str">
         <f aca="false">IF(A9="","",IF(MAX(V9,AF9)&lt;=0,"Pass",IF(V9&gt;=AF9,"Flip","Value-add hold")))</f>
-        <v/>
-      </c>
-      <c r="D9" s="23" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D9" s="23" t="n">
         <f aca="false">IF(A9="","",MAX(V9,AF9))</f>
-        <v/>
+        <v>151838.39663286</v>
       </c>
       <c r="E9" s="24" t="str">
         <f aca="false">IF(A9="","",IF(D9&lt;=0,"Pass",IF(N(Deals!D9)&lt;=1,"$1 = awaiting minimum bid; re-check the morning of Nov 3",IF(D9&lt;Deals!D9,"Max bid below opening bid: pass","Room of "&amp;TEXT(D9-Deals!D9,"$#,##0")&amp;" over opening bid"))))</f>
-        <v/>
-      </c>
-      <c r="F9" s="23" t="str">
+        <v>Room of $124,638 over opening bid</v>
+      </c>
+      <c r="F9" s="23" t="n">
         <f aca="false">IF(A9="","",IF(C9="Flip",W9,IF(C9="Value-add hold",AG9,0)))</f>
-        <v/>
+        <v>480234.705882353</v>
       </c>
       <c r="G9" s="24" t="str">
         <f aca="false">IF(A9="","",IF(C9="Flip",TEXT(X9,"$#,##0")&amp;" profit, "&amp;TEXT(Y9,"0%")&amp;"/yr over "&amp;TEXT(M9,"0")&amp;" mo",IF(C9="Value-add hold",TEXT(AH9,"0.0%")&amp;" yield on cost; "&amp;IF(ISNUMBER(AJ9),TEXT(AJ9,"0.0%")&amp;" cash-on-cash after refi","all cash out at refi"),"")))</f>
-        <v/>
+        <v>$132,065 profit, 15%/yr over 22 mo</v>
       </c>
       <c r="H9" s="21" t="str">
         <f aca="false">IF(A9="","",IF(C9="Flip",IF(W9&lt;=FlipCeiling,"In $300k flip box","Over flip ceiling: needs to be exceptional"),IF(C9="Value-add hold","Value-add","")))</f>
-        <v/>
+        <v>Over flip ceiling: needs to be exceptional</v>
       </c>
       <c r="I9" s="24" t="str">
         <f aca="false">IF(A9="","",TRIM(IF(AK9&gt;D9,"Wholesale assignment supports "&amp;TEXT(AK9,"$#,##0")&amp;". ","")&amp;IF(AND(ISNUMBER(AN9),N(AN9)&gt;D9),"Teardown/new units supports "&amp;TEXT(AN9,"$#,##0")&amp;".","")))</f>
-        <v/>
+        <v>Wholesale assignment supports $167,419.</v>
       </c>
       <c r="J9" s="24" t="str">
         <f aca="false">IF(A9="","",TRIM(IF(Deals!F9="2nd","Plaintiff is 2nd: add senior mortgage to surviving liens. ",IF(Deals!F9&lt;&gt;"1st","Lien position unconfirmed. ",""))&amp;IF(N(Deals!M9)=0,"No ARV yet. ","")&amp;IF(N(Deals!G9)=0,"No building sf: rehab is allowance only. ","")&amp;IF(AND(N(Deals!S9)&gt;0,D9&gt;0,D9*(1-RTTPurchase)-SheriffCostsFromBid&lt;N(Deals!S9)),"City claims not fully paid at max bid; unpaid part is counted as cost. ","")&amp;IF(K9=1,"Occupancy assumed: +"&amp;TEXT(EjectMonths,"0")&amp;" mo and possession cost. ","")))</f>
         <v/>
       </c>
-      <c r="K9" s="22" t="str">
+      <c r="K9" s="22" t="n">
         <f aca="false">IF(A9="","",IF(OR(Deals!Q9="Occupied",AND(Deals!Q9&lt;&gt;"Vacant",UnknownAsOccupied="Y")),1,0))</f>
-        <v/>
-      </c>
-      <c r="L9" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="L9" s="25" t="n">
         <f aca="false">IF(A9="","",IFERROR(INDEX(ScopeMonths,MATCH(Deals!O9,ScopeNames,0)),INDEX(ScopeMonths,3)))</f>
-        <v/>
-      </c>
-      <c r="M9" s="25" t="str">
+        <v>7</v>
+      </c>
+      <c r="M9" s="25" t="n">
         <f aca="false">IF(A9="","",DeedMonths+K9*EjectMonths+L9+SellMonths)</f>
-        <v/>
-      </c>
-      <c r="N9" s="25" t="str">
+        <v>22</v>
+      </c>
+      <c r="N9" s="25" t="n">
         <f aca="false">IF(A9="","",DeedMonths+K9*EjectMonths+L9+LeaseUpMonths)</f>
-        <v/>
-      </c>
-      <c r="O9" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="O9" s="26" t="n">
         <f aca="false">IF(A9="","",N(Deals!G9)*IFERROR(INDEX(ScopePSF,MATCH(Deals!O9,ScopeNames,0)),INDEX(ScopePSF,3))*(1+Contingency)+BlindAllowance+N(Deals!P9))</f>
-        <v/>
-      </c>
-      <c r="P9" s="26" t="str">
+        <v>299200</v>
+      </c>
+      <c r="P9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(N(Deals!K9)&gt;0,Deals!K9,N(Deals!M9))*TaxRate/12+VacantInsMo+SecuringMo+UtilitiesMo+N(Deals!T9))</f>
-        <v/>
-      </c>
-      <c r="Q9" s="26" t="str">
+        <v>902.21515</v>
+      </c>
+      <c r="Q9" s="26" t="n">
         <f aca="false">IF(A9="","",SheriffFees+PurchaseTitle+CompelDeedLegal+K9*PossessionCost+N(Deals!R9)+N(Deals!T9)*HOAArrearsMonths)</f>
-        <v/>
-      </c>
-      <c r="R9" s="26" t="str">
+        <v>7070</v>
+      </c>
+      <c r="R9" s="26" t="n">
         <f aca="false">IF(A9="","",N(Deals!M9)*(BrokerPct+SellerRTT+SellClosingPct+ConcessionsPct))</f>
-        <v/>
-      </c>
-      <c r="S9" s="26" t="str">
+        <v>62700.75</v>
+      </c>
+      <c r="S9" s="26" t="n">
         <f aca="false">IF(A9="","",Q9+O9+P9*M9)</f>
-        <v/>
-      </c>
-      <c r="T9" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="T9" s="26" t="n">
         <f aca="false">IF(A9="","",N(Deals!M9)-R9-S9)</f>
-        <v/>
-      </c>
-      <c r="U9" s="26" t="str">
+        <v>286180.5167</v>
+      </c>
+      <c r="U9" s="26" t="n">
         <f aca="false">IF(A9="","",MIN(T9-FlipTarget,(T9-FlipMinAnnROI*M9/12*S9)/(1+FlipMinAnnROI*M9/12)))</f>
-        <v/>
-      </c>
-      <c r="V9" s="26" t="str">
+        <v>154115.972582353</v>
+      </c>
+      <c r="V9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(N(Deals!S9)=0,MAX(0,(U9)/(1+BuyerPremium)),IF((U9)&gt;=(N(Deals!S9)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(U9)/(1+BuyerPremium),MAX(0,((U9)-N(Deals!S9)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="W9" s="26" t="str">
+        <v>151838.39663286</v>
+      </c>
+      <c r="W9" s="26" t="n">
         <f aca="false">IF(A9="","",((V9)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(V9)*(1-RTTPurchase)))))+S9)</f>
-        <v/>
-      </c>
-      <c r="X9" s="26" t="str">
+        <v>480234.705882353</v>
+      </c>
+      <c r="X9" s="26" t="n">
         <f aca="false">IF(A9="","",T9-((V9)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(V9)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="Y9" s="27" t="str">
+        <v>132064.544117647</v>
+      </c>
+      <c r="Y9" s="27" t="n">
         <f aca="false">IF(A9="","",IFERROR(X9/W9/(M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="Z9" s="26" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="Z9" s="26" t="n">
         <f aca="false">IF(A9="","",N(Deals!N9)*12*(1-Vacancy)*(1-MgmtPct-MaintPct-CapexPct)-N(Deals!M9)*TaxRate-MAX(1,N(Deals!J9))*(InsPerUnit+WaterPerUnit)-N(Deals!T9)*12)</f>
-        <v/>
-      </c>
-      <c r="AA9" s="26" t="str">
+        <v>17220.95</v>
+      </c>
+      <c r="AA9" s="26" t="n">
         <f aca="false">IF(A9="","",Q9+O9+P9*N9)</f>
-        <v/>
-      </c>
-      <c r="AB9" s="26" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AB9" s="26" t="n">
         <f aca="false">IF(A9="","",MAX(0,MIN(RefiLTV*N(Deals!M9),Z9/(RefiDSCR*12*PMT(RefiRate/12,RefiTerm*12,-1)))))</f>
-        <v/>
-      </c>
-      <c r="AC9" s="26" t="str">
+        <v>175306.491960853</v>
+      </c>
+      <c r="AC9" s="26" t="n">
         <f aca="false">IF(A9="","",Z9-AB9*12*PMT(RefiRate/12,RefiTerm*12,-1))</f>
-        <v/>
-      </c>
-      <c r="AD9" s="26" t="str">
+        <v>2870.15833333333</v>
+      </c>
+      <c r="AD9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(N(Deals!S9)=0,MAX(0,(Z9/HoldTarget-AA9)/(1+BuyerPremium)),IF((Z9/HoldTarget-AA9)&gt;=(N(Deals!S9)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(Z9/HoldTarget-AA9)/(1+BuyerPremium),MAX(0,((Z9/HoldTarget-AA9)-N(Deals!S9)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="AE9" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(AC9&lt;=0,0,IF(N(Deals!S9)=0,MAX(0,(AC9/HoldTarget+AB9*(1-RefiCostPct)-AA9)/(1+BuyerPremium)),IF((AC9/HoldTarget+AB9*(1-RefiCostPct)-AA9)&gt;=(N(Deals!S9)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(AC9/HoldTarget+AB9*(1-RefiCostPct)-AA9)/(1+BuyerPremium),MAX(0,((AC9/HoldTarget+AB9*(1-RefiCostPct)-AA9)-N(Deals!S9)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF9" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(HoldMeasure="Cash-on-cash",AE9,AD9))</f>
-        <v/>
-      </c>
-      <c r="AG9" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="26" t="n">
         <f aca="false">IF(A9="","",((AF9)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AF9)*(1-RTTPurchase)))))+AA9)</f>
-        <v/>
-      </c>
-      <c r="AH9" s="27" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AH9" s="27" t="n">
         <f aca="false">IF(A9="","",IFERROR(Z9/AG9,0))</f>
-        <v/>
-      </c>
-      <c r="AI9" s="26" t="str">
+        <v>0.0529522611519295</v>
+      </c>
+      <c r="AI9" s="26" t="n">
         <f aca="false">IF(A9="","",AG9-AB9*(1-RefiCostPct))</f>
-        <v/>
-      </c>
-      <c r="AJ9" s="27" t="str">
+        <v>155169.220947972</v>
+      </c>
+      <c r="AJ9" s="27" t="n">
         <f aca="false">IF(A9="","",IF(AI9&lt;=0,"All cash out",AC9/AI9))</f>
-        <v/>
-      </c>
-      <c r="AK9" s="26" t="str">
+        <v>0.0184969565213947</v>
+      </c>
+      <c r="AK9" s="26" t="n">
         <f aca="false">IF(A9="","",IF(N(Deals!S9)=0,MAX(0,(T9-BuyerMarginPct*N(Deals!M9)-WholesaleMinFee)/(1+BuyerPremium)),IF((T9-BuyerMarginPct*N(Deals!M9)-WholesaleMinFee)&gt;=(N(Deals!S9)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(T9-BuyerMarginPct*N(Deals!M9)-WholesaleMinFee)/(1+BuyerPremium),MAX(0,((T9-BuyerMarginPct*N(Deals!M9)-WholesaleMinFee)-N(Deals!S9)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
+        <v>167419.228275862</v>
       </c>
       <c r="AL9" s="26" t="str">
         <f aca="false">IF(OR(A9="",N(Deals!U9)=0),"",Deals!U9*N(Deals!W9))</f>
@@ -5244,154 +5420,154 @@
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="str">
         <f aca="false">IF(Deals!A10="","",Deals!A10)</f>
-        <v/>
+        <v>1311511-7</v>
       </c>
       <c r="B10" s="0" t="str">
         <f aca="false">IF(A10="","",Deals!B10)</f>
-        <v/>
+        <v>7 Gut + $30k foundation, ARV 640k, vacant</v>
       </c>
       <c r="C10" s="21" t="str">
         <f aca="false">IF(A10="","",IF(MAX(V10,AF10)&lt;=0,"Pass",IF(V10&gt;=AF10,"Flip","Value-add hold")))</f>
-        <v/>
-      </c>
-      <c r="D10" s="23" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D10" s="23" t="n">
         <f aca="false">IF(A10="","",MAX(V10,AF10))</f>
-        <v/>
+        <v>127305.333752536</v>
       </c>
       <c r="E10" s="24" t="str">
         <f aca="false">IF(A10="","",IF(D10&lt;=0,"Pass",IF(N(Deals!D10)&lt;=1,"$1 = awaiting minimum bid; re-check the morning of Nov 3",IF(D10&lt;Deals!D10,"Max bid below opening bid: pass","Room of "&amp;TEXT(D10-Deals!D10,"$#,##0")&amp;" over opening bid"))))</f>
-        <v/>
-      </c>
-      <c r="F10" s="23" t="str">
+        <v>Room of $100,105 over opening bid</v>
+      </c>
+      <c r="F10" s="23" t="n">
         <f aca="false">IF(A10="","",IF(C10="Flip",W10,IF(C10="Value-add hold",AG10,0)))</f>
-        <v/>
+        <v>455333.647058824</v>
       </c>
       <c r="G10" s="24" t="str">
         <f aca="false">IF(A10="","",IF(C10="Flip",TEXT(X10,"$#,##0")&amp;" profit, "&amp;TEXT(Y10,"0%")&amp;"/yr over "&amp;TEXT(M10,"0")&amp;" mo",IF(C10="Value-add hold",TEXT(AH10,"0.0%")&amp;" yield on cost; "&amp;IF(ISNUMBER(AJ10),TEXT(AJ10,"0.0%")&amp;" cash-on-cash after refi","all cash out at refi"),"")))</f>
-        <v/>
+        <v>$125,217 profit, 15%/yr over 22 mo</v>
       </c>
       <c r="H10" s="21" t="str">
         <f aca="false">IF(A10="","",IF(C10="Flip",IF(W10&lt;=FlipCeiling,"In $300k flip box","Over flip ceiling: needs to be exceptional"),IF(C10="Value-add hold","Value-add","")))</f>
-        <v/>
+        <v>Over flip ceiling: needs to be exceptional</v>
       </c>
       <c r="I10" s="24" t="str">
         <f aca="false">IF(A10="","",TRIM(IF(AK10&gt;D10,"Wholesale assignment supports "&amp;TEXT(AK10,"$#,##0")&amp;". ","")&amp;IF(AND(ISNUMBER(AN10),N(AN10)&gt;D10),"Teardown/new units supports "&amp;TEXT(AN10,"$#,##0")&amp;".","")))</f>
-        <v/>
+        <v>Wholesale assignment supports $141,312.</v>
       </c>
       <c r="J10" s="24" t="str">
         <f aca="false">IF(A10="","",TRIM(IF(Deals!F10="2nd","Plaintiff is 2nd: add senior mortgage to surviving liens. ",IF(Deals!F10&lt;&gt;"1st","Lien position unconfirmed. ",""))&amp;IF(N(Deals!M10)=0,"No ARV yet. ","")&amp;IF(N(Deals!G10)=0,"No building sf: rehab is allowance only. ","")&amp;IF(AND(N(Deals!S10)&gt;0,D10&gt;0,D10*(1-RTTPurchase)-SheriffCostsFromBid&lt;N(Deals!S10)),"City claims not fully paid at max bid; unpaid part is counted as cost. ","")&amp;IF(K10=1,"Occupancy assumed: +"&amp;TEXT(EjectMonths,"0")&amp;" mo and possession cost. ","")))</f>
         <v/>
       </c>
-      <c r="K10" s="22" t="str">
+      <c r="K10" s="22" t="n">
         <f aca="false">IF(A10="","",IF(OR(Deals!Q10="Occupied",AND(Deals!Q10&lt;&gt;"Vacant",UnknownAsOccupied="Y")),1,0))</f>
-        <v/>
-      </c>
-      <c r="L10" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="L10" s="25" t="n">
         <f aca="false">IF(A10="","",IFERROR(INDEX(ScopeMonths,MATCH(Deals!O10,ScopeNames,0)),INDEX(ScopeMonths,3)))</f>
-        <v/>
-      </c>
-      <c r="M10" s="25" t="str">
+        <v>7</v>
+      </c>
+      <c r="M10" s="25" t="n">
         <f aca="false">IF(A10="","",DeedMonths+K10*EjectMonths+L10+SellMonths)</f>
-        <v/>
-      </c>
-      <c r="N10" s="25" t="str">
+        <v>22</v>
+      </c>
+      <c r="N10" s="25" t="n">
         <f aca="false">IF(A10="","",DeedMonths+K10*EjectMonths+L10+LeaseUpMonths)</f>
-        <v/>
-      </c>
-      <c r="O10" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="O10" s="26" t="n">
         <f aca="false">IF(A10="","",N(Deals!G10)*IFERROR(INDEX(ScopePSF,MATCH(Deals!O10,ScopeNames,0)),INDEX(ScopePSF,3))*(1+Contingency)+BlindAllowance+N(Deals!P10))</f>
-        <v/>
-      </c>
-      <c r="P10" s="26" t="str">
+        <v>299200</v>
+      </c>
+      <c r="P10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(N(Deals!K10)&gt;0,Deals!K10,N(Deals!M10))*TaxRate/12+VacantInsMo+SecuringMo+UtilitiesMo+N(Deals!T10))</f>
-        <v/>
-      </c>
-      <c r="Q10" s="26" t="str">
+        <v>902.21515</v>
+      </c>
+      <c r="Q10" s="26" t="n">
         <f aca="false">IF(A10="","",SheriffFees+PurchaseTitle+CompelDeedLegal+K10*PossessionCost+N(Deals!R10)+N(Deals!T10)*HOAArrearsMonths)</f>
-        <v/>
-      </c>
-      <c r="R10" s="26" t="str">
+        <v>7070</v>
+      </c>
+      <c r="R10" s="26" t="n">
         <f aca="false">IF(A10="","",N(Deals!M10)*(BrokerPct+SellerRTT+SellClosingPct+ConcessionsPct))</f>
-        <v/>
-      </c>
-      <c r="S10" s="26" t="str">
+        <v>59449.6</v>
+      </c>
+      <c r="S10" s="26" t="n">
         <f aca="false">IF(A10="","",Q10+O10+P10*M10)</f>
-        <v/>
-      </c>
-      <c r="T10" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="T10" s="26" t="n">
         <f aca="false">IF(A10="","",N(Deals!M10)-R10-S10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="26" t="str">
+        <v>254431.6667</v>
+      </c>
+      <c r="U10" s="26" t="n">
         <f aca="false">IF(A10="","",MIN(T10-FlipTarget,(T10-FlipMinAnnROI*M10/12*S10)/(1+FlipMinAnnROI*M10/12)))</f>
-        <v/>
-      </c>
-      <c r="V10" s="26" t="str">
+        <v>129214.913758824</v>
+      </c>
+      <c r="V10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(N(Deals!S10)=0,MAX(0,(U10)/(1+BuyerPremium)),IF((U10)&gt;=(N(Deals!S10)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(U10)/(1+BuyerPremium),MAX(0,((U10)-N(Deals!S10)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="W10" s="26" t="str">
+        <v>127305.333752536</v>
+      </c>
+      <c r="W10" s="26" t="n">
         <f aca="false">IF(A10="","",((V10)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(V10)*(1-RTTPurchase)))))+S10)</f>
-        <v/>
-      </c>
-      <c r="X10" s="26" t="str">
+        <v>455333.647058824</v>
+      </c>
+      <c r="X10" s="26" t="n">
         <f aca="false">IF(A10="","",T10-((V10)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(V10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="Y10" s="27" t="str">
+        <v>125216.752941176</v>
+      </c>
+      <c r="Y10" s="27" t="n">
         <f aca="false">IF(A10="","",IFERROR(X10/W10/(M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="Z10" s="26" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="Z10" s="26" t="n">
         <f aca="false">IF(A10="","",N(Deals!N10)*12*(1-Vacancy)*(1-MgmtPct-MaintPct-CapexPct)-N(Deals!M10)*TaxRate-MAX(1,N(Deals!J10))*(InsPerUnit+WaterPerUnit)-N(Deals!T10)*12)</f>
-        <v/>
-      </c>
-      <c r="AA10" s="26" t="str">
+        <v>17710.88</v>
+      </c>
+      <c r="AA10" s="26" t="n">
         <f aca="false">IF(A10="","",Q10+O10+P10*N10)</f>
-        <v/>
-      </c>
-      <c r="AB10" s="26" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AB10" s="26" t="n">
         <f aca="false">IF(A10="","",MAX(0,MIN(RefiLTV*N(Deals!M10),Z10/(RefiDSCR*12*PMT(RefiRate/12,RefiTerm*12,-1)))))</f>
-        <v/>
-      </c>
-      <c r="AC10" s="26" t="str">
+        <v>180293.900298162</v>
+      </c>
+      <c r="AC10" s="26" t="n">
         <f aca="false">IF(A10="","",Z10-AB10*12*PMT(RefiRate/12,RefiTerm*12,-1))</f>
-        <v/>
-      </c>
-      <c r="AD10" s="26" t="str">
+        <v>2951.81333333334</v>
+      </c>
+      <c r="AD10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(N(Deals!S10)=0,MAX(0,(Z10/HoldTarget-AA10)/(1+BuyerPremium)),IF((Z10/HoldTarget-AA10)&gt;=(N(Deals!S10)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(Z10/HoldTarget-AA10)/(1+BuyerPremium),MAX(0,((Z10/HoldTarget-AA10)-N(Deals!S10)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="AE10" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(AC10&lt;=0,0,IF(N(Deals!S10)=0,MAX(0,(AC10/HoldTarget+AB10*(1-RefiCostPct)-AA10)/(1+BuyerPremium)),IF((AC10/HoldTarget+AB10*(1-RefiCostPct)-AA10)&gt;=(N(Deals!S10)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(AC10/HoldTarget+AB10*(1-RefiCostPct)-AA10)/(1+BuyerPremium),MAX(0,((AC10/HoldTarget+AB10*(1-RefiCostPct)-AA10)-N(Deals!S10)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF10" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(HoldMeasure="Cash-on-cash",AE10,AD10))</f>
-        <v/>
-      </c>
-      <c r="AG10" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="26" t="n">
         <f aca="false">IF(A10="","",((AF10)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AF10)*(1-RTTPurchase)))))+AA10)</f>
-        <v/>
-      </c>
-      <c r="AH10" s="27" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AH10" s="27" t="n">
         <f aca="false">IF(A10="","",IFERROR(Z10/AG10,0))</f>
-        <v/>
-      </c>
-      <c r="AI10" s="26" t="str">
+        <v>0.0544587344478954</v>
+      </c>
+      <c r="AI10" s="26" t="n">
         <f aca="false">IF(A10="","",AG10-AB10*(1-RefiCostPct))</f>
-        <v/>
-      </c>
-      <c r="AJ10" s="27" t="str">
+        <v>150331.434860783</v>
+      </c>
+      <c r="AJ10" s="27" t="n">
         <f aca="false">IF(A10="","",IF(AI10&lt;=0,"All cash out",AC10/AI10))</f>
-        <v/>
-      </c>
-      <c r="AK10" s="26" t="str">
+        <v>0.0196353699149278</v>
+      </c>
+      <c r="AK10" s="26" t="n">
         <f aca="false">IF(A10="","",IF(N(Deals!S10)=0,MAX(0,(T10-BuyerMarginPct*N(Deals!M10)-WholesaleMinFee)/(1+BuyerPremium)),IF((T10-BuyerMarginPct*N(Deals!M10)-WholesaleMinFee)&gt;=(N(Deals!S10)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(T10-BuyerMarginPct*N(Deals!M10)-WholesaleMinFee)/(1+BuyerPremium),MAX(0,((T10-BuyerMarginPct*N(Deals!M10)-WholesaleMinFee)-N(Deals!S10)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
+        <v>141311.986896552</v>
       </c>
       <c r="AL10" s="26" t="str">
         <f aca="false">IF(OR(A10="",N(Deals!U10)=0),"",Deals!U10*N(Deals!W10))</f>
@@ -5406,154 +5582,154 @@
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="str">
         <f aca="false">IF(Deals!A11="","",Deals!A11)</f>
-        <v/>
+        <v>1311511-8</v>
       </c>
       <c r="B11" s="0" t="str">
         <f aca="false">IF(A11="","",Deals!B11)</f>
-        <v/>
+        <v>8 Gut + $30k foundation, ARV 710k, vacant</v>
       </c>
       <c r="C11" s="21" t="str">
         <f aca="false">IF(A11="","",IF(MAX(V11,AF11)&lt;=0,"Pass",IF(V11&gt;=AF11,"Flip","Value-add hold")))</f>
-        <v/>
-      </c>
-      <c r="D11" s="23" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D11" s="23" t="n">
         <f aca="false">IF(A11="","",MAX(V11,AF11))</f>
-        <v/>
+        <v>176371.459513185</v>
       </c>
       <c r="E11" s="24" t="str">
         <f aca="false">IF(A11="","",IF(D11&lt;=0,"Pass",IF(N(Deals!D11)&lt;=1,"$1 = awaiting minimum bid; re-check the morning of Nov 3",IF(D11&lt;Deals!D11,"Max bid below opening bid: pass","Room of "&amp;TEXT(D11-Deals!D11,"$#,##0")&amp;" over opening bid"))))</f>
-        <v/>
-      </c>
-      <c r="F11" s="23" t="str">
+        <v>Room of $149,171 over opening bid</v>
+      </c>
+      <c r="F11" s="23" t="n">
         <f aca="false">IF(A11="","",IF(C11="Flip",W11,IF(C11="Value-add hold",AG11,0)))</f>
-        <v/>
+        <v>505135.764705882</v>
       </c>
       <c r="G11" s="24" t="str">
         <f aca="false">IF(A11="","",IF(C11="Flip",TEXT(X11,"$#,##0")&amp;" profit, "&amp;TEXT(Y11,"0%")&amp;"/yr over "&amp;TEXT(M11,"0")&amp;" mo",IF(C11="Value-add hold",TEXT(AH11,"0.0%")&amp;" yield on cost; "&amp;IF(ISNUMBER(AJ11),TEXT(AJ11,"0.0%")&amp;" cash-on-cash after refi","all cash out at refi"),"")))</f>
-        <v/>
+        <v>$138,912 profit, 15%/yr over 22 mo</v>
       </c>
       <c r="H11" s="21" t="str">
         <f aca="false">IF(A11="","",IF(C11="Flip",IF(W11&lt;=FlipCeiling,"In $300k flip box","Over flip ceiling: needs to be exceptional"),IF(C11="Value-add hold","Value-add","")))</f>
-        <v/>
+        <v>Over flip ceiling: needs to be exceptional</v>
       </c>
       <c r="I11" s="24" t="str">
         <f aca="false">IF(A11="","",TRIM(IF(AK11&gt;D11,"Wholesale assignment supports "&amp;TEXT(AK11,"$#,##0")&amp;". ","")&amp;IF(AND(ISNUMBER(AN11),N(AN11)&gt;D11),"Teardown/new units supports "&amp;TEXT(AN11,"$#,##0")&amp;".","")))</f>
-        <v/>
+        <v>Wholesale assignment supports $193,526.</v>
       </c>
       <c r="J11" s="24" t="str">
         <f aca="false">IF(A11="","",TRIM(IF(Deals!F11="2nd","Plaintiff is 2nd: add senior mortgage to surviving liens. ",IF(Deals!F11&lt;&gt;"1st","Lien position unconfirmed. ",""))&amp;IF(N(Deals!M11)=0,"No ARV yet. ","")&amp;IF(N(Deals!G11)=0,"No building sf: rehab is allowance only. ","")&amp;IF(AND(N(Deals!S11)&gt;0,D11&gt;0,D11*(1-RTTPurchase)-SheriffCostsFromBid&lt;N(Deals!S11)),"City claims not fully paid at max bid; unpaid part is counted as cost. ","")&amp;IF(K11=1,"Occupancy assumed: +"&amp;TEXT(EjectMonths,"0")&amp;" mo and possession cost. ","")))</f>
         <v/>
       </c>
-      <c r="K11" s="22" t="str">
+      <c r="K11" s="22" t="n">
         <f aca="false">IF(A11="","",IF(OR(Deals!Q11="Occupied",AND(Deals!Q11&lt;&gt;"Vacant",UnknownAsOccupied="Y")),1,0))</f>
-        <v/>
-      </c>
-      <c r="L11" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="L11" s="25" t="n">
         <f aca="false">IF(A11="","",IFERROR(INDEX(ScopeMonths,MATCH(Deals!O11,ScopeNames,0)),INDEX(ScopeMonths,3)))</f>
-        <v/>
-      </c>
-      <c r="M11" s="25" t="str">
+        <v>7</v>
+      </c>
+      <c r="M11" s="25" t="n">
         <f aca="false">IF(A11="","",DeedMonths+K11*EjectMonths+L11+SellMonths)</f>
-        <v/>
-      </c>
-      <c r="N11" s="25" t="str">
+        <v>22</v>
+      </c>
+      <c r="N11" s="25" t="n">
         <f aca="false">IF(A11="","",DeedMonths+K11*EjectMonths+L11+LeaseUpMonths)</f>
-        <v/>
-      </c>
-      <c r="O11" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="O11" s="26" t="n">
         <f aca="false">IF(A11="","",N(Deals!G11)*IFERROR(INDEX(ScopePSF,MATCH(Deals!O11,ScopeNames,0)),INDEX(ScopePSF,3))*(1+Contingency)+BlindAllowance+N(Deals!P11))</f>
-        <v/>
-      </c>
-      <c r="P11" s="26" t="str">
+        <v>299200</v>
+      </c>
+      <c r="P11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(N(Deals!K11)&gt;0,Deals!K11,N(Deals!M11))*TaxRate/12+VacantInsMo+SecuringMo+UtilitiesMo+N(Deals!T11))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="26" t="str">
+        <v>902.21515</v>
+      </c>
+      <c r="Q11" s="26" t="n">
         <f aca="false">IF(A11="","",SheriffFees+PurchaseTitle+CompelDeedLegal+K11*PossessionCost+N(Deals!R11)+N(Deals!T11)*HOAArrearsMonths)</f>
-        <v/>
-      </c>
-      <c r="R11" s="26" t="str">
+        <v>7070</v>
+      </c>
+      <c r="R11" s="26" t="n">
         <f aca="false">IF(A11="","",N(Deals!M11)*(BrokerPct+SellerRTT+SellClosingPct+ConcessionsPct))</f>
-        <v/>
-      </c>
-      <c r="S11" s="26" t="str">
+        <v>65951.9</v>
+      </c>
+      <c r="S11" s="26" t="n">
         <f aca="false">IF(A11="","",Q11+O11+P11*M11)</f>
-        <v/>
-      </c>
-      <c r="T11" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="T11" s="26" t="n">
         <f aca="false">IF(A11="","",N(Deals!M11)-R11-S11)</f>
-        <v/>
-      </c>
-      <c r="U11" s="26" t="str">
+        <v>317929.3667</v>
+      </c>
+      <c r="U11" s="26" t="n">
         <f aca="false">IF(A11="","",MIN(T11-FlipTarget,(T11-FlipMinAnnROI*M11/12*S11)/(1+FlipMinAnnROI*M11/12)))</f>
-        <v/>
-      </c>
-      <c r="V11" s="26" t="str">
+        <v>179017.031405882</v>
+      </c>
+      <c r="V11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(N(Deals!S11)=0,MAX(0,(U11)/(1+BuyerPremium)),IF((U11)&gt;=(N(Deals!S11)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(U11)/(1+BuyerPremium),MAX(0,((U11)-N(Deals!S11)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="W11" s="26" t="str">
+        <v>176371.459513185</v>
+      </c>
+      <c r="W11" s="26" t="n">
         <f aca="false">IF(A11="","",((V11)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(V11)*(1-RTTPurchase)))))+S11)</f>
-        <v/>
-      </c>
-      <c r="X11" s="26" t="str">
+        <v>505135.764705882</v>
+      </c>
+      <c r="X11" s="26" t="n">
         <f aca="false">IF(A11="","",T11-((V11)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(V11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="Y11" s="27" t="str">
+        <v>138912.335294118</v>
+      </c>
+      <c r="Y11" s="27" t="n">
         <f aca="false">IF(A11="","",IFERROR(X11/W11/(M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="Z11" s="26" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="Z11" s="26" t="n">
         <f aca="false">IF(A11="","",N(Deals!N11)*12*(1-Vacancy)*(1-MgmtPct-MaintPct-CapexPct)-N(Deals!M11)*TaxRate-MAX(1,N(Deals!J11))*(InsPerUnit+WaterPerUnit)-N(Deals!T11)*12)</f>
-        <v/>
-      </c>
-      <c r="AA11" s="26" t="str">
+        <v>16731.02</v>
+      </c>
+      <c r="AA11" s="26" t="n">
         <f aca="false">IF(A11="","",Q11+O11+P11*N11)</f>
-        <v/>
-      </c>
-      <c r="AB11" s="26" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AB11" s="26" t="n">
         <f aca="false">IF(A11="","",MAX(0,MIN(RefiLTV*N(Deals!M11),Z11/(RefiDSCR*12*PMT(RefiRate/12,RefiTerm*12,-1)))))</f>
-        <v/>
-      </c>
-      <c r="AC11" s="26" t="str">
+        <v>170319.083623544</v>
+      </c>
+      <c r="AC11" s="26" t="n">
         <f aca="false">IF(A11="","",Z11-AB11*12*PMT(RefiRate/12,RefiTerm*12,-1))</f>
-        <v/>
-      </c>
-      <c r="AD11" s="26" t="str">
+        <v>2788.50333333334</v>
+      </c>
+      <c r="AD11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(N(Deals!S11)=0,MAX(0,(Z11/HoldTarget-AA11)/(1+BuyerPremium)),IF((Z11/HoldTarget-AA11)&gt;=(N(Deals!S11)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(Z11/HoldTarget-AA11)/(1+BuyerPremium),MAX(0,((Z11/HoldTarget-AA11)-N(Deals!S11)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="AE11" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(AC11&lt;=0,0,IF(N(Deals!S11)=0,MAX(0,(AC11/HoldTarget+AB11*(1-RefiCostPct)-AA11)/(1+BuyerPremium)),IF((AC11/HoldTarget+AB11*(1-RefiCostPct)-AA11)&gt;=(N(Deals!S11)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(AC11/HoldTarget+AB11*(1-RefiCostPct)-AA11)/(1+BuyerPremium),MAX(0,((AC11/HoldTarget+AB11*(1-RefiCostPct)-AA11)-N(Deals!S11)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF11" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(HoldMeasure="Cash-on-cash",AE11,AD11))</f>
-        <v/>
-      </c>
-      <c r="AG11" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AG11" s="26" t="n">
         <f aca="false">IF(A11="","",((AF11)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AF11)*(1-RTTPurchase)))))+AA11)</f>
-        <v/>
-      </c>
-      <c r="AH11" s="27" t="str">
+        <v>325216.51815</v>
+      </c>
+      <c r="AH11" s="27" t="n">
         <f aca="false">IF(A11="","",IFERROR(Z11/AG11,0))</f>
-        <v/>
-      </c>
-      <c r="AI11" s="26" t="str">
+        <v>0.0514457878559635</v>
+      </c>
+      <c r="AI11" s="26" t="n">
         <f aca="false">IF(A11="","",AG11-AB11*(1-RefiCostPct))</f>
-        <v/>
-      </c>
-      <c r="AJ11" s="27" t="str">
+        <v>160007.007035162</v>
+      </c>
+      <c r="AJ11" s="27" t="n">
         <f aca="false">IF(A11="","",IF(AI11&lt;=0,"All cash out",AC11/AI11))</f>
-        <v/>
-      </c>
-      <c r="AK11" s="26" t="str">
+        <v>0.0174273826190659</v>
+      </c>
+      <c r="AK11" s="26" t="n">
         <f aca="false">IF(A11="","",IF(N(Deals!S11)=0,MAX(0,(T11-BuyerMarginPct*N(Deals!M11)-WholesaleMinFee)/(1+BuyerPremium)),IF((T11-BuyerMarginPct*N(Deals!M11)-WholesaleMinFee)&gt;=(N(Deals!S11)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(T11-BuyerMarginPct*N(Deals!M11)-WholesaleMinFee)/(1+BuyerPremium),MAX(0,((T11-BuyerMarginPct*N(Deals!M11)-WholesaleMinFee)-N(Deals!S11)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
+        <v>193526.469655172</v>
       </c>
       <c r="AL11" s="26" t="str">
         <f aca="false">IF(OR(A11="",N(Deals!U11)=0),"",Deals!U11*N(Deals!W11))</f>
@@ -5568,154 +5744,154 @@
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="str">
         <f aca="false">IF(Deals!A12="","",Deals!A12)</f>
-        <v/>
+        <v>1311511-9</v>
       </c>
       <c r="B12" s="0" t="str">
         <f aca="false">IF(A12="","",Deals!B12)</f>
-        <v/>
+        <v>9 Gut + $30k foundation, ARV 675k, + $15k estate/title cure</v>
       </c>
       <c r="C12" s="21" t="str">
         <f aca="false">IF(A12="","",IF(MAX(V12,AF12)&lt;=0,"Pass",IF(V12&gt;=AF12,"Flip","Value-add hold")))</f>
-        <v/>
-      </c>
-      <c r="D12" s="23" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D12" s="23" t="n">
         <f aca="false">IF(A12="","",MAX(V12,AF12))</f>
-        <v/>
+        <v>137060.071509707</v>
       </c>
       <c r="E12" s="24" t="str">
         <f aca="false">IF(A12="","",IF(D12&lt;=0,"Pass",IF(N(Deals!D12)&lt;=1,"$1 = awaiting minimum bid; re-check the morning of Nov 3",IF(D12&lt;Deals!D12,"Max bid below opening bid: pass","Room of "&amp;TEXT(D12-Deals!D12,"$#,##0")&amp;" over opening bid"))))</f>
-        <v/>
-      </c>
-      <c r="F12" s="23" t="str">
+        <v>Room of $109,860 over opening bid</v>
+      </c>
+      <c r="F12" s="23" t="n">
         <f aca="false">IF(A12="","",IF(C12="Flip",W12,IF(C12="Value-add hold",AG12,0)))</f>
-        <v/>
+        <v>480234.705882353</v>
       </c>
       <c r="G12" s="24" t="str">
         <f aca="false">IF(A12="","",IF(C12="Flip",TEXT(X12,"$#,##0")&amp;" profit, "&amp;TEXT(Y12,"0%")&amp;"/yr over "&amp;TEXT(M12,"0")&amp;" mo",IF(C12="Value-add hold",TEXT(AH12,"0.0%")&amp;" yield on cost; "&amp;IF(ISNUMBER(AJ12),TEXT(AJ12,"0.0%")&amp;" cash-on-cash after refi","all cash out at refi"),"")))</f>
-        <v/>
+        <v>$132,065 profit, 15%/yr over 22 mo</v>
       </c>
       <c r="H12" s="21" t="str">
         <f aca="false">IF(A12="","",IF(C12="Flip",IF(W12&lt;=FlipCeiling,"In $300k flip box","Over flip ceiling: needs to be exceptional"),IF(C12="Value-add hold","Value-add","")))</f>
-        <v/>
+        <v>Over flip ceiling: needs to be exceptional</v>
       </c>
       <c r="I12" s="24" t="str">
         <f aca="false">IF(A12="","",TRIM(IF(AK12&gt;D12,"Wholesale assignment supports "&amp;TEXT(AK12,"$#,##0")&amp;". ","")&amp;IF(AND(ISNUMBER(AN12),N(AN12)&gt;D12),"Teardown/new units supports "&amp;TEXT(AN12,"$#,##0")&amp;".","")))</f>
-        <v/>
+        <v>Wholesale assignment supports $152,641.</v>
       </c>
       <c r="J12" s="24" t="str">
         <f aca="false">IF(A12="","",TRIM(IF(Deals!F12="2nd","Plaintiff is 2nd: add senior mortgage to surviving liens. ",IF(Deals!F12&lt;&gt;"1st","Lien position unconfirmed. ",""))&amp;IF(N(Deals!M12)=0,"No ARV yet. ","")&amp;IF(N(Deals!G12)=0,"No building sf: rehab is allowance only. ","")&amp;IF(AND(N(Deals!S12)&gt;0,D12&gt;0,D12*(1-RTTPurchase)-SheriffCostsFromBid&lt;N(Deals!S12)),"City claims not fully paid at max bid; unpaid part is counted as cost. ","")&amp;IF(K12=1,"Occupancy assumed: +"&amp;TEXT(EjectMonths,"0")&amp;" mo and possession cost. ","")))</f>
         <v/>
       </c>
-      <c r="K12" s="22" t="str">
+      <c r="K12" s="22" t="n">
         <f aca="false">IF(A12="","",IF(OR(Deals!Q12="Occupied",AND(Deals!Q12&lt;&gt;"Vacant",UnknownAsOccupied="Y")),1,0))</f>
-        <v/>
-      </c>
-      <c r="L12" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="L12" s="25" t="n">
         <f aca="false">IF(A12="","",IFERROR(INDEX(ScopeMonths,MATCH(Deals!O12,ScopeNames,0)),INDEX(ScopeMonths,3)))</f>
-        <v/>
-      </c>
-      <c r="M12" s="25" t="str">
+        <v>7</v>
+      </c>
+      <c r="M12" s="25" t="n">
         <f aca="false">IF(A12="","",DeedMonths+K12*EjectMonths+L12+SellMonths)</f>
-        <v/>
-      </c>
-      <c r="N12" s="25" t="str">
+        <v>22</v>
+      </c>
+      <c r="N12" s="25" t="n">
         <f aca="false">IF(A12="","",DeedMonths+K12*EjectMonths+L12+LeaseUpMonths)</f>
-        <v/>
-      </c>
-      <c r="O12" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="O12" s="26" t="n">
         <f aca="false">IF(A12="","",N(Deals!G12)*IFERROR(INDEX(ScopePSF,MATCH(Deals!O12,ScopeNames,0)),INDEX(ScopePSF,3))*(1+Contingency)+BlindAllowance+N(Deals!P12))</f>
-        <v/>
-      </c>
-      <c r="P12" s="26" t="str">
+        <v>299200</v>
+      </c>
+      <c r="P12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(N(Deals!K12)&gt;0,Deals!K12,N(Deals!M12))*TaxRate/12+VacantInsMo+SecuringMo+UtilitiesMo+N(Deals!T12))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="26" t="str">
+        <v>902.21515</v>
+      </c>
+      <c r="Q12" s="26" t="n">
         <f aca="false">IF(A12="","",SheriffFees+PurchaseTitle+CompelDeedLegal+K12*PossessionCost+N(Deals!R12)+N(Deals!T12)*HOAArrearsMonths)</f>
-        <v/>
-      </c>
-      <c r="R12" s="26" t="str">
+        <v>22070</v>
+      </c>
+      <c r="R12" s="26" t="n">
         <f aca="false">IF(A12="","",N(Deals!M12)*(BrokerPct+SellerRTT+SellClosingPct+ConcessionsPct))</f>
-        <v/>
-      </c>
-      <c r="S12" s="26" t="str">
+        <v>62700.75</v>
+      </c>
+      <c r="S12" s="26" t="n">
         <f aca="false">IF(A12="","",Q12+O12+P12*M12)</f>
-        <v/>
-      </c>
-      <c r="T12" s="26" t="str">
+        <v>341118.7333</v>
+      </c>
+      <c r="T12" s="26" t="n">
         <f aca="false">IF(A12="","",N(Deals!M12)-R12-S12)</f>
-        <v/>
-      </c>
-      <c r="U12" s="26" t="str">
+        <v>271180.5167</v>
+      </c>
+      <c r="U12" s="26" t="n">
         <f aca="false">IF(A12="","",MIN(T12-FlipTarget,(T12-FlipMinAnnROI*M12/12*S12)/(1+FlipMinAnnROI*M12/12)))</f>
-        <v/>
-      </c>
-      <c r="V12" s="26" t="str">
+        <v>139115.972582353</v>
+      </c>
+      <c r="V12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(N(Deals!S12)=0,MAX(0,(U12)/(1+BuyerPremium)),IF((U12)&gt;=(N(Deals!S12)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(U12)/(1+BuyerPremium),MAX(0,((U12)-N(Deals!S12)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="W12" s="26" t="str">
+        <v>137060.071509707</v>
+      </c>
+      <c r="W12" s="26" t="n">
         <f aca="false">IF(A12="","",((V12)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(V12)*(1-RTTPurchase)))))+S12)</f>
-        <v/>
-      </c>
-      <c r="X12" s="26" t="str">
+        <v>480234.705882353</v>
+      </c>
+      <c r="X12" s="26" t="n">
         <f aca="false">IF(A12="","",T12-((V12)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(V12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="Y12" s="27" t="str">
+        <v>132064.544117647</v>
+      </c>
+      <c r="Y12" s="27" t="n">
         <f aca="false">IF(A12="","",IFERROR(X12/W12/(M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="Z12" s="26" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="Z12" s="26" t="n">
         <f aca="false">IF(A12="","",N(Deals!N12)*12*(1-Vacancy)*(1-MgmtPct-MaintPct-CapexPct)-N(Deals!M12)*TaxRate-MAX(1,N(Deals!J12))*(InsPerUnit+WaterPerUnit)-N(Deals!T12)*12)</f>
-        <v/>
-      </c>
-      <c r="AA12" s="26" t="str">
+        <v>17220.95</v>
+      </c>
+      <c r="AA12" s="26" t="n">
         <f aca="false">IF(A12="","",Q12+O12+P12*N12)</f>
-        <v/>
-      </c>
-      <c r="AB12" s="26" t="str">
+        <v>340216.51815</v>
+      </c>
+      <c r="AB12" s="26" t="n">
         <f aca="false">IF(A12="","",MAX(0,MIN(RefiLTV*N(Deals!M12),Z12/(RefiDSCR*12*PMT(RefiRate/12,RefiTerm*12,-1)))))</f>
-        <v/>
-      </c>
-      <c r="AC12" s="26" t="str">
+        <v>175306.491960853</v>
+      </c>
+      <c r="AC12" s="26" t="n">
         <f aca="false">IF(A12="","",Z12-AB12*12*PMT(RefiRate/12,RefiTerm*12,-1))</f>
-        <v/>
-      </c>
-      <c r="AD12" s="26" t="str">
+        <v>2870.15833333333</v>
+      </c>
+      <c r="AD12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(N(Deals!S12)=0,MAX(0,(Z12/HoldTarget-AA12)/(1+BuyerPremium)),IF((Z12/HoldTarget-AA12)&gt;=(N(Deals!S12)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(Z12/HoldTarget-AA12)/(1+BuyerPremium),MAX(0,((Z12/HoldTarget-AA12)-N(Deals!S12)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
-      </c>
-      <c r="AE12" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(AC12&lt;=0,0,IF(N(Deals!S12)=0,MAX(0,(AC12/HoldTarget+AB12*(1-RefiCostPct)-AA12)/(1+BuyerPremium)),IF((AC12/HoldTarget+AB12*(1-RefiCostPct)-AA12)&gt;=(N(Deals!S12)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(AC12/HoldTarget+AB12*(1-RefiCostPct)-AA12)/(1+BuyerPremium),MAX(0,((AC12/HoldTarget+AB12*(1-RefiCostPct)-AA12)-N(Deals!S12)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF12" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(HoldMeasure="Cash-on-cash",AE12,AD12))</f>
-        <v/>
-      </c>
-      <c r="AG12" s="26" t="str">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="26" t="n">
         <f aca="false">IF(A12="","",((AF12)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AF12)*(1-RTTPurchase)))))+AA12)</f>
-        <v/>
-      </c>
-      <c r="AH12" s="27" t="str">
+        <v>340216.51815</v>
+      </c>
+      <c r="AH12" s="27" t="n">
         <f aca="false">IF(A12="","",IFERROR(Z12/AG12,0))</f>
-        <v/>
-      </c>
-      <c r="AI12" s="26" t="str">
+        <v>0.0506176187259884</v>
+      </c>
+      <c r="AI12" s="26" t="n">
         <f aca="false">IF(A12="","",AG12-AB12*(1-RefiCostPct))</f>
-        <v/>
-      </c>
-      <c r="AJ12" s="27" t="str">
+        <v>170169.220947972</v>
+      </c>
+      <c r="AJ12" s="27" t="n">
         <f aca="false">IF(A12="","",IF(AI12&lt;=0,"All cash out",AC12/AI12))</f>
-        <v/>
-      </c>
-      <c r="AK12" s="26" t="str">
+        <v>0.0168664951120089</v>
+      </c>
+      <c r="AK12" s="26" t="n">
         <f aca="false">IF(A12="","",IF(N(Deals!S12)=0,MAX(0,(T12-BuyerMarginPct*N(Deals!M12)-WholesaleMinFee)/(1+BuyerPremium)),IF((T12-BuyerMarginPct*N(Deals!M12)-WholesaleMinFee)&gt;=(N(Deals!S12)+SheriffCostsFromBid)/(1-RTTPurchase)*(1+BuyerPremium),(T12-BuyerMarginPct*N(Deals!M12)-WholesaleMinFee)/(1+BuyerPremium),MAX(0,((T12-BuyerMarginPct*N(Deals!M12)-WholesaleMinFee)-N(Deals!S12)-SheriffCostsFromBid)/(BuyerPremium+RTTPurchase)))))</f>
-        <v/>
+        <v>152640.903152709</v>
       </c>
       <c r="AL12" s="26" t="str">
         <f aca="false">IF(OR(A12="",N(Deals!U12)=0),"",Deals!U12*N(Deals!W12))</f>
@@ -10616,12 +10792,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F2" s="18" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="J2" s="28" t="n">
         <v>0.2</v>
@@ -10642,7 +10818,7 @@
         <v>0.7</v>
       </c>
       <c r="AH2" s="18" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10659,103 +10835,103 @@
         <v>131</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="AD3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="AE3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="AF3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="AG3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="AH3" s="5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="AI3" s="5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="AJ3" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="AK3" s="5" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11661,601 +11837,601 @@
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="str">
         <f aca="false">Underwriting!$A9</f>
-        <v/>
+        <v>1311511-6</v>
       </c>
       <c r="B10" s="0" t="str">
         <f aca="false">Underwriting!$B9</f>
-        <v/>
-      </c>
-      <c r="C10" s="26" t="str">
+        <v>6 Gut + $30k foundation, ARV 675k, vacant</v>
+      </c>
+      <c r="C10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",N(Deals!M9))</f>
-        <v/>
-      </c>
-      <c r="D10" s="26" t="str">
+        <v>675000</v>
+      </c>
+      <c r="D10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",N(Deals!D9))</f>
-        <v/>
-      </c>
-      <c r="E10" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="E10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$D9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="26" t="str">
+        <v>151838.39663286</v>
+      </c>
+      <c r="F10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",$D10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="G10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((F10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(F10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="H10" s="27" t="str">
+        <v>258572.5167</v>
+      </c>
+      <c r="H10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(G10/(((F10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(F10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="I10" s="27" t="str">
+        <v>0.398724612210802</v>
+      </c>
+      <c r="I10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((F10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(F10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="J10" s="26" t="str">
+        <v>0.0488088245405856</v>
+      </c>
+      <c r="J10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(J$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="K10" s="26" t="str">
+        <v>135000</v>
+      </c>
+      <c r="K10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((J10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(J10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="L10" s="27" t="str">
+        <v>149155.5167</v>
+      </c>
+      <c r="L10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(K10/(((J10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(J10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="M10" s="27" t="str">
+        <v>0.175663727508404</v>
+      </c>
+      <c r="M10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((J10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(J10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="N10" s="26" t="str">
+        <v>0.0372553077207827</v>
+      </c>
+      <c r="N10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(N$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="O10" s="26" t="str">
+        <v>203000</v>
+      </c>
+      <c r="O10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((N10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="P10" s="27" t="str">
+        <v>80135.5167</v>
+      </c>
+      <c r="P10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(O10/(((N10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="Q10" s="27" t="str">
+        <v>0.0821369046802793</v>
+      </c>
+      <c r="Q10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((N10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="R10" s="26" t="str">
+        <v>0.0324152030810892</v>
+      </c>
+      <c r="R10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(R$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="S10" s="26" t="str">
+        <v>270000</v>
+      </c>
+      <c r="S10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((R10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(R10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="T10" s="27" t="str">
+        <v>12130.5167</v>
+      </c>
+      <c r="T10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(S10/(((R10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(R10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="U10" s="27" t="str">
+        <v>0.0110246420808127</v>
+      </c>
+      <c r="U10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((R10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(R10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="V10" s="26" t="str">
+        <v>0.0287367130958074</v>
+      </c>
+      <c r="V10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(V$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="W10" s="26" t="str">
+        <v>338000</v>
+      </c>
+      <c r="W10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((V10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(V10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="X10" s="27" t="str">
+        <v>-56889.4833</v>
+      </c>
+      <c r="X10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(W10/(((V10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(V10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="Y10" s="27" t="str">
+        <v>-0.0463705165828521</v>
+      </c>
+      <c r="Y10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((V10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(V10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="Z10" s="26" t="str">
+        <v>0.0257688125262085</v>
+      </c>
+      <c r="Z10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(Z$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="AA10" s="26" t="str">
+        <v>405000</v>
+      </c>
+      <c r="AA10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((Z10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(Z10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AB10" s="27" t="str">
+        <v>-124894.4833</v>
+      </c>
+      <c r="AB10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(AA10/(((Z10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(Z10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="AC10" s="27" t="str">
+        <v>-0.0924102587161559</v>
+      </c>
+      <c r="AC10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((Z10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(Z10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="AD10" s="26" t="str">
+        <v>0.0233887659649662</v>
+      </c>
+      <c r="AD10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",ROUND(AD$2*$C10,-3))</f>
-        <v/>
-      </c>
-      <c r="AE10" s="26" t="str">
+        <v>473000</v>
+      </c>
+      <c r="AE10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((AD10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AD10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF10" s="27" t="str">
+        <v>-193914.4833</v>
+      </c>
+      <c r="AF10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(AE10/(((AD10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AD10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="AG10" s="27" t="str">
+        <v>-0.131195403869529</v>
+      </c>
+      <c r="AG10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((AD10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AD10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
-      </c>
-      <c r="AH10" s="26" t="str">
+        <v>0.0213842092306848</v>
+      </c>
+      <c r="AH10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",$E10)</f>
-        <v/>
-      </c>
-      <c r="AI10" s="26" t="str">
+        <v>151838.39663286</v>
+      </c>
+      <c r="AI10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$T9-((AH10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AH10)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AJ10" s="27" t="str">
+        <v>132064.544117647</v>
+      </c>
+      <c r="AJ10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(AI10/(((AH10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AH10)*(1-RTTPurchase)))))+Underwriting!$S9)/(Underwriting!$M9/12),0))</f>
-        <v/>
-      </c>
-      <c r="AK10" s="27" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="AK10" s="27" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IFERROR(Underwriting!$Z9/(((AH10)*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(AH10)*(1-RTTPurchase)))))+Underwriting!$AA9),0))</f>
-        <v/>
+        <v>0.0359269407623272</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="str">
         <f aca="false">Underwriting!$A10</f>
-        <v/>
+        <v>1311511-7</v>
       </c>
       <c r="B11" s="0" t="str">
         <f aca="false">Underwriting!$B10</f>
-        <v/>
-      </c>
-      <c r="C11" s="26" t="str">
+        <v>7 Gut + $30k foundation, ARV 640k, vacant</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",N(Deals!M10))</f>
-        <v/>
-      </c>
-      <c r="D11" s="26" t="str">
+        <v>640000</v>
+      </c>
+      <c r="D11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",N(Deals!D10))</f>
-        <v/>
-      </c>
-      <c r="E11" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="E11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$D10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="26" t="str">
+        <v>127305.333752536</v>
+      </c>
+      <c r="F11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",$D11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="G11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((F11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(F11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="H11" s="27" t="str">
+        <v>226823.6667</v>
+      </c>
+      <c r="H11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(G11/(((F11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(F11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="I11" s="27" t="str">
+        <v>0.349767174405932</v>
+      </c>
+      <c r="I11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((F11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(F11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="J11" s="26" t="str">
+        <v>0.0501974185152019</v>
+      </c>
+      <c r="J11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(J$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="K11" s="26" t="str">
+        <v>128000</v>
+      </c>
+      <c r="K11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((J11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(J11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="L11" s="27" t="str">
+        <v>124511.6667</v>
+      </c>
+      <c r="L11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(K11/(((J11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(J11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="M11" s="27" t="str">
+        <v>0.148924750474997</v>
+      </c>
+      <c r="M11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((J11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(J11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="N11" s="26" t="str">
+        <v>0.0389133354361229</v>
+      </c>
+      <c r="N11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(N$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="O11" s="26" t="str">
+        <v>192000</v>
+      </c>
+      <c r="O11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((N11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="P11" s="27" t="str">
+        <v>59551.6667</v>
+      </c>
+      <c r="P11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(O11/(((N11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="27" t="str">
+        <v>0.0623470369786965</v>
+      </c>
+      <c r="Q11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((N11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="R11" s="26" t="str">
+        <v>0.0340530639639699</v>
+      </c>
+      <c r="R11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(R$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="S11" s="26" t="str">
+        <v>256000</v>
+      </c>
+      <c r="S11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((R11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(R11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="T11" s="27" t="str">
+        <v>-5408.33329999997</v>
+      </c>
+      <c r="T11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(S11/(((R11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(R11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="U11" s="27" t="str">
+        <v>-0.0050344841951657</v>
+      </c>
+      <c r="U11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((R11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(R11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="V11" s="26" t="str">
+        <v>0.0302720838937123</v>
+      </c>
+      <c r="V11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(V$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="W11" s="26" t="str">
+        <v>320000</v>
+      </c>
+      <c r="W11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((V11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(V11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="X11" s="27" t="str">
+        <v>-70368.3332999999</v>
+      </c>
+      <c r="X11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(W11/(((V11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(V11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="Y11" s="27" t="str">
+        <v>-0.0589670035458256</v>
+      </c>
+      <c r="Y11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((V11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(V11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="Z11" s="26" t="str">
+        <v>0.0272468152815664</v>
+      </c>
+      <c r="Z11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(Z$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="AA11" s="26" t="str">
+        <v>384000</v>
+      </c>
+      <c r="AA11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((Z11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(Z11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AB11" s="27" t="str">
+        <v>-135328.3333</v>
+      </c>
+      <c r="AB11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(AA11/(((Z11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(Z11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="AC11" s="27" t="str">
+        <v>-0.103111673938132</v>
+      </c>
+      <c r="AC11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((Z11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(Z11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="AD11" s="26" t="str">
+        <v>0.0247712750704413</v>
+      </c>
+      <c r="AD11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",ROUND(AD$2*$C11,-3))</f>
-        <v/>
-      </c>
-      <c r="AE11" s="26" t="str">
+        <v>448000</v>
+      </c>
+      <c r="AE11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((AD11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AD11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF11" s="27" t="str">
+        <v>-200288.3333</v>
+      </c>
+      <c r="AF11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(AE11/(((AD11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AD11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="AG11" s="27" t="str">
+        <v>-0.139911325016233</v>
+      </c>
+      <c r="AG11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((AD11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AD11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
-      </c>
-      <c r="AH11" s="26" t="str">
+        <v>0.0227081045544707</v>
+      </c>
+      <c r="AH11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",$E11)</f>
-        <v/>
-      </c>
-      <c r="AI11" s="26" t="str">
+        <v>127305.333752536</v>
+      </c>
+      <c r="AI11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$T10-((AH11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AH11)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AJ11" s="27" t="str">
+        <v>125216.752941176</v>
+      </c>
+      <c r="AJ11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(AI11/(((AH11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AH11)*(1-RTTPurchase)))))+Underwriting!$S10)/(Underwriting!$M10/12),0))</f>
-        <v/>
-      </c>
-      <c r="AK11" s="27" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="AK11" s="27" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IFERROR(Underwriting!$Z10/(((AH11)*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(AH11)*(1-RTTPurchase)))))+Underwriting!$AA10),0))</f>
-        <v/>
+        <v>0.0389737125480209</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="str">
         <f aca="false">Underwriting!$A11</f>
-        <v/>
+        <v>1311511-8</v>
       </c>
       <c r="B12" s="0" t="str">
         <f aca="false">Underwriting!$B11</f>
-        <v/>
-      </c>
-      <c r="C12" s="26" t="str">
+        <v>8 Gut + $30k foundation, ARV 710k, vacant</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",N(Deals!M11))</f>
-        <v/>
-      </c>
-      <c r="D12" s="26" t="str">
+        <v>710000</v>
+      </c>
+      <c r="D12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",N(Deals!D11))</f>
-        <v/>
-      </c>
-      <c r="E12" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="E12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$D11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="26" t="str">
+        <v>176371.459513185</v>
+      </c>
+      <c r="F12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",$D12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="G12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((F12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(F12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="H12" s="27" t="str">
+        <v>290321.3667</v>
+      </c>
+      <c r="H12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(G12/(((F12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(F12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="I12" s="27" t="str">
+        <v>0.447682050015672</v>
+      </c>
+      <c r="I12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((F12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(F12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="J12" s="26" t="str">
+        <v>0.0474202305659693</v>
+      </c>
+      <c r="J12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(J$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="K12" s="26" t="str">
+        <v>142000</v>
+      </c>
+      <c r="K12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((J12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(J12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="L12" s="27" t="str">
+        <v>173799.3667</v>
+      </c>
+      <c r="L12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(K12/(((J12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(J12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="M12" s="27" t="str">
+        <v>0.201594704781816</v>
+      </c>
+      <c r="M12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((J12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(J12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="N12" s="26" t="str">
+        <v>0.0356474786815248</v>
+      </c>
+      <c r="N12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(N$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="O12" s="26" t="str">
+        <v>213000</v>
+      </c>
+      <c r="O12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((N12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="P12" s="27" t="str">
+        <v>101734.3667</v>
+      </c>
+      <c r="P12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(O12/(((N12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="27" t="str">
+        <v>0.102323561691471</v>
+      </c>
+      <c r="Q12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((N12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="R12" s="26" t="str">
+        <v>0.0309025933862098</v>
+      </c>
+      <c r="R12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(R$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="S12" s="26" t="str">
+        <v>284000</v>
+      </c>
+      <c r="S12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((R12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(R12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="T12" s="27" t="str">
+        <v>29669.3667</v>
+      </c>
+      <c r="T12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(S12/(((R12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(R12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="U12" s="27" t="str">
+        <v>0.026340903501571</v>
+      </c>
+      <c r="U12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((R12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(R12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="V12" s="26" t="str">
+        <v>0.0272724701027744</v>
+      </c>
+      <c r="V12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(V$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="W12" s="26" t="str">
+        <v>355000</v>
+      </c>
+      <c r="W12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((V12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(V12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="X12" s="27" t="str">
+        <v>-42395.6333</v>
+      </c>
+      <c r="X12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(W12/(((V12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(V12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="Y12" s="27" t="str">
+        <v>-0.0336879627114357</v>
+      </c>
+      <c r="Y12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((V12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(V12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="Z12" s="26" t="str">
+        <v>0.0244055532116425</v>
+      </c>
+      <c r="Z12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(Z$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="AA12" s="26" t="str">
+        <v>426000</v>
+      </c>
+      <c r="AA12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((Z12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(Z12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AB12" s="27" t="str">
+        <v>-114460.6333</v>
+      </c>
+      <c r="AB12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(AA12/(((Z12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(Z12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="AC12" s="27" t="str">
+        <v>-0.0823102885545786</v>
+      </c>
+      <c r="AC12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((Z12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(Z12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="AD12" s="26" t="str">
+        <v>0.0220840497001735</v>
+      </c>
+      <c r="AD12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",ROUND(AD$2*$C12,-3))</f>
-        <v/>
-      </c>
-      <c r="AE12" s="26" t="str">
+        <v>497000</v>
+      </c>
+      <c r="AE12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((AD12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AD12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF12" s="27" t="str">
+        <v>-186525.6333</v>
+      </c>
+      <c r="AF12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(AE12/(((AD12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AD12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="AG12" s="27" t="str">
+        <v>-0.122495150578671</v>
+      </c>
+      <c r="AG12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((AD12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AD12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
-      </c>
-      <c r="AH12" s="26" t="str">
+        <v>0.0201658362785634</v>
+      </c>
+      <c r="AH12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",$E12)</f>
-        <v/>
-      </c>
-      <c r="AI12" s="26" t="str">
+        <v>176371.459513185</v>
+      </c>
+      <c r="AI12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$T11-((AH12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AH12)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AJ12" s="27" t="str">
+        <v>138912.335294118</v>
+      </c>
+      <c r="AJ12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(AI12/(((AH12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AH12)*(1-RTTPurchase)))))+Underwriting!$S11)/(Underwriting!$M11/12),0))</f>
-        <v/>
-      </c>
-      <c r="AK12" s="27" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="AK12" s="27" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IFERROR(Underwriting!$Z11/(((AH12)*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(AH12)*(1-RTTPurchase)))))+Underwriting!$AA11),0))</f>
-        <v/>
+        <v>0.0331810924019957</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="str">
         <f aca="false">Underwriting!$A12</f>
-        <v/>
+        <v>1311511-9</v>
       </c>
       <c r="B13" s="0" t="str">
         <f aca="false">Underwriting!$B12</f>
-        <v/>
-      </c>
-      <c r="C13" s="26" t="str">
+        <v>9 Gut + $30k foundation, ARV 675k, + $15k estate/title cure</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",N(Deals!M12))</f>
-        <v/>
-      </c>
-      <c r="D13" s="26" t="str">
+        <v>675000</v>
+      </c>
+      <c r="D13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",N(Deals!D12))</f>
-        <v/>
-      </c>
-      <c r="E13" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="E13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$D12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="26" t="str">
+        <v>137060.071509707</v>
+      </c>
+      <c r="F13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",$D13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="26" t="str">
+        <v>27200</v>
+      </c>
+      <c r="G13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((F13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(F13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="H13" s="27" t="str">
+        <v>243572.5167</v>
+      </c>
+      <c r="H13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(G13/(((F13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(F13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="I13" s="27" t="str">
+        <v>0.360314900937014</v>
+      </c>
+      <c r="I13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((F13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(F13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="J13" s="26" t="str">
+        <v>0.0468183852632065</v>
+      </c>
+      <c r="J13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(J$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="K13" s="26" t="str">
+        <v>135000</v>
+      </c>
+      <c r="K13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((J13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(J13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="L13" s="27" t="str">
+        <v>134155.5167</v>
+      </c>
+      <c r="L13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(K13/(((J13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(J13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="M13" s="27" t="str">
+        <v>0.153041295504977</v>
+      </c>
+      <c r="M13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((J13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(J13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="N13" s="26" t="str">
+        <v>0.036084350051429</v>
+      </c>
+      <c r="N13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(N$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="O13" s="26" t="str">
+        <v>203000</v>
+      </c>
+      <c r="O13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((N13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="P13" s="27" t="str">
+        <v>65135.5167</v>
+      </c>
+      <c r="P13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(O13/(((N13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="Q13" s="27" t="str">
+        <v>0.0649320513994407</v>
+      </c>
+      <c r="Q13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((N13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="R13" s="26" t="str">
+        <v>0.0315251018565639</v>
+      </c>
+      <c r="R13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(R$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="S13" s="26" t="str">
+        <v>270000</v>
+      </c>
+      <c r="S13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((R13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(R13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="T13" s="27" t="str">
+        <v>-2869.48330000002</v>
+      </c>
+      <c r="T13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(S13/(((R13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(R13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="U13" s="27" t="str">
+        <v>-0.00254429821342632</v>
+      </c>
+      <c r="U13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((R13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(R13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="V13" s="26" t="str">
+        <v>0.0280349807309451</v>
+      </c>
+      <c r="V13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(V$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="W13" s="26" t="str">
+        <v>338000</v>
+      </c>
+      <c r="W13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((V13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(V13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="X13" s="27" t="str">
+        <v>-71889.4833</v>
+      </c>
+      <c r="X13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(W13/(((V13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(V13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="Y13" s="27" t="str">
+        <v>-0.0573123226499696</v>
+      </c>
+      <c r="Y13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((V13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(V13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="Z13" s="26" t="str">
+        <v>0.0252031169100567</v>
+      </c>
+      <c r="Z13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(Z$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="AA13" s="26" t="str">
+        <v>405000</v>
+      </c>
+      <c r="AA13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((Z13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(Z13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AB13" s="27" t="str">
+        <v>-139894.4833</v>
+      </c>
+      <c r="AB13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(AA13/(((Z13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(Z13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="AC13" s="27" t="str">
+        <v>-0.101444718856181</v>
+      </c>
+      <c r="AC13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((Z13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(Z13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="AD13" s="26" t="str">
+        <v>0.0229217947813458</v>
+      </c>
+      <c r="AD13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",ROUND(AD$2*$C13,-3))</f>
-        <v/>
-      </c>
-      <c r="AE13" s="26" t="str">
+        <v>473000</v>
+      </c>
+      <c r="AE13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((AD13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AD13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AF13" s="27" t="str">
+        <v>-208914.4833</v>
+      </c>
+      <c r="AF13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(AE13/(((AD13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AD13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="AG13" s="27" t="str">
+        <v>-0.13876211503351</v>
+      </c>
+      <c r="AG13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((AD13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AD13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
-      </c>
-      <c r="AH13" s="26" t="str">
+        <v>0.020993183222439</v>
+      </c>
+      <c r="AH13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",$E13)</f>
-        <v/>
-      </c>
-      <c r="AI13" s="26" t="str">
+        <v>137060.071509707</v>
+      </c>
+      <c r="AI13" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$T12-((AH13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AH13)*(1-RTTPurchase))))))</f>
-        <v/>
-      </c>
-      <c r="AJ13" s="27" t="str">
+        <v>132064.544117647</v>
+      </c>
+      <c r="AJ13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(AI13/(((AH13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AH13)*(1-RTTPurchase)))))+Underwriting!$S12)/(Underwriting!$M12/12),0))</f>
-        <v/>
-      </c>
-      <c r="AK13" s="27" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="AK13" s="27" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IFERROR(Underwriting!$Z12/(((AH13)*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(AH13)*(1-RTTPurchase)))))+Underwriting!$AA12),0))</f>
-        <v/>
+        <v>0.0359269407623272</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16785,7 +16961,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16796,34 +16972,34 @@
         <v>129</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17129,201 +17305,201 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="str">
         <f aca="false">Underwriting!$A9</f>
-        <v/>
+        <v>1311511-6</v>
       </c>
       <c r="B9" s="0" t="str">
         <f aca="false">Underwriting!$B9</f>
-        <v/>
+        <v>6 Gut + $30k foundation, ARV 675k, vacant</v>
       </c>
       <c r="C9" s="0" t="str">
         <f aca="false">Underwriting!$C9</f>
-        <v/>
-      </c>
-      <c r="D9" s="26" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D9" s="26" t="n">
         <f aca="false">Underwriting!$D9</f>
-        <v/>
-      </c>
-      <c r="E9" s="8" t="str">
+        <v>151838.39663286</v>
+      </c>
+      <c r="E9" s="8" t="n">
         <f aca="false">IF(Underwriting!$A9="","",Underwriting!$D9)</f>
-        <v/>
+        <v>151838.39663286</v>
       </c>
       <c r="F9" s="11" t="str">
         <f aca="false">IF(Underwriting!$A9="","",IF(Underwriting!$D9&gt;0,"Y","N"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="26" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G9" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",N(E9)*(DownPct+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="H9" s="26" t="str">
+        <v>17461.4156127789</v>
+      </c>
+      <c r="H9" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IF(N(E9)&gt;0,N(E9)*(1-DownPct)+35,0))</f>
-        <v/>
-      </c>
-      <c r="I9" s="26" t="str">
+        <v>136689.556969574</v>
+      </c>
+      <c r="I9" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",IF(C9="Value-add hold",Underwriting!$AA9,Underwriting!$S9)+((N(E9))*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N(E9))*(1-RTTPurchase)))))-N(E9)*(1+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="J9" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="J9" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",G9+H9+I9)</f>
-        <v/>
-      </c>
-      <c r="K9" s="26" t="str">
+        <v>480269.705882353</v>
+      </c>
+      <c r="K9" s="26" t="n">
         <f aca="false">IF(Underwriting!$A9="","",SUMIF($F$3:F9,"Y",$J$3:J9))</f>
-        <v/>
+        <v>2897033.20936281</v>
       </c>
       <c r="L9" s="0" t="str">
         <f aca="false">IF(Underwriting!$A9="","",IF(C9="Value-add hold",TEXT(IFERROR(Underwriting!$Z9/(((N(E9))*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N(E9))*(1-RTTPurchase)))))+Underwriting!$AA9),0),"0.0%")&amp;" yield on cost",TEXT(Underwriting!$T9-((N(E9))*(1+BuyerPremium)+IF(N(Deals!S9)=0,0,MIN(N(Deals!S9),MAX(0,N(Deals!S9)+SheriffCostsFromBid-(N(E9))*(1-RTTPurchase))))),"$#,##0")&amp;" flip profit"))</f>
-        <v/>
+        <v>$132,065 flip profit</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="str">
         <f aca="false">Underwriting!$A10</f>
-        <v/>
+        <v>1311511-7</v>
       </c>
       <c r="B10" s="0" t="str">
         <f aca="false">Underwriting!$B10</f>
-        <v/>
+        <v>7 Gut + $30k foundation, ARV 640k, vacant</v>
       </c>
       <c r="C10" s="0" t="str">
         <f aca="false">Underwriting!$C10</f>
-        <v/>
-      </c>
-      <c r="D10" s="26" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D10" s="26" t="n">
         <f aca="false">Underwriting!$D10</f>
-        <v/>
-      </c>
-      <c r="E10" s="8" t="str">
+        <v>127305.333752536</v>
+      </c>
+      <c r="E10" s="8" t="n">
         <f aca="false">IF(Underwriting!$A10="","",Underwriting!$D10)</f>
-        <v/>
+        <v>127305.333752536</v>
       </c>
       <c r="F10" s="11" t="str">
         <f aca="false">IF(Underwriting!$A10="","",IF(Underwriting!$D10&gt;0,"Y","N"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="26" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",N(E10)*(DownPct+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="H10" s="26" t="str">
+        <v>14640.1133815416</v>
+      </c>
+      <c r="H10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IF(N(E10)&gt;0,N(E10)*(1-DownPct)+35,0))</f>
-        <v/>
-      </c>
-      <c r="I10" s="26" t="str">
+        <v>114609.800377282</v>
+      </c>
+      <c r="I10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",IF(C10="Value-add hold",Underwriting!$AA10,Underwriting!$S10)+((N(E10))*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N(E10))*(1-RTTPurchase)))))-N(E10)*(1+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="J10" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="J10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",G10+H10+I10)</f>
-        <v/>
-      </c>
-      <c r="K10" s="26" t="str">
+        <v>455368.647058824</v>
+      </c>
+      <c r="K10" s="26" t="n">
         <f aca="false">IF(Underwriting!$A10="","",SUMIF($F$3:F10,"Y",$J$3:J10))</f>
-        <v/>
+        <v>3352401.85642164</v>
       </c>
       <c r="L10" s="0" t="str">
         <f aca="false">IF(Underwriting!$A10="","",IF(C10="Value-add hold",TEXT(IFERROR(Underwriting!$Z10/(((N(E10))*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N(E10))*(1-RTTPurchase)))))+Underwriting!$AA10),0),"0.0%")&amp;" yield on cost",TEXT(Underwriting!$T10-((N(E10))*(1+BuyerPremium)+IF(N(Deals!S10)=0,0,MIN(N(Deals!S10),MAX(0,N(Deals!S10)+SheriffCostsFromBid-(N(E10))*(1-RTTPurchase))))),"$#,##0")&amp;" flip profit"))</f>
-        <v/>
+        <v>$125,217 flip profit</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="str">
         <f aca="false">Underwriting!$A11</f>
-        <v/>
+        <v>1311511-8</v>
       </c>
       <c r="B11" s="0" t="str">
         <f aca="false">Underwriting!$B11</f>
-        <v/>
+        <v>8 Gut + $30k foundation, ARV 710k, vacant</v>
       </c>
       <c r="C11" s="0" t="str">
         <f aca="false">Underwriting!$C11</f>
-        <v/>
-      </c>
-      <c r="D11" s="26" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D11" s="26" t="n">
         <f aca="false">Underwriting!$D11</f>
-        <v/>
-      </c>
-      <c r="E11" s="8" t="str">
+        <v>176371.459513185</v>
+      </c>
+      <c r="E11" s="8" t="n">
         <f aca="false">IF(Underwriting!$A11="","",Underwriting!$D11)</f>
-        <v/>
+        <v>176371.459513185</v>
       </c>
       <c r="F11" s="11" t="str">
         <f aca="false">IF(Underwriting!$A11="","",IF(Underwriting!$D11&gt;0,"Y","N"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="26" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",N(E11)*(DownPct+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="H11" s="26" t="str">
+        <v>20282.7178440162</v>
+      </c>
+      <c r="H11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IF(N(E11)&gt;0,N(E11)*(1-DownPct)+35,0))</f>
-        <v/>
-      </c>
-      <c r="I11" s="26" t="str">
+        <v>158769.313561866</v>
+      </c>
+      <c r="I11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",IF(C11="Value-add hold",Underwriting!$AA11,Underwriting!$S11)+((N(E11))*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N(E11))*(1-RTTPurchase)))))-N(E11)*(1+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="J11" s="26" t="str">
+        <v>326118.7333</v>
+      </c>
+      <c r="J11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",G11+H11+I11)</f>
-        <v/>
-      </c>
-      <c r="K11" s="26" t="str">
+        <v>505170.764705882</v>
+      </c>
+      <c r="K11" s="26" t="n">
         <f aca="false">IF(Underwriting!$A11="","",SUMIF($F$3:F11,"Y",$J$3:J11))</f>
-        <v/>
+        <v>3857572.62112752</v>
       </c>
       <c r="L11" s="0" t="str">
         <f aca="false">IF(Underwriting!$A11="","",IF(C11="Value-add hold",TEXT(IFERROR(Underwriting!$Z11/(((N(E11))*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N(E11))*(1-RTTPurchase)))))+Underwriting!$AA11),0),"0.0%")&amp;" yield on cost",TEXT(Underwriting!$T11-((N(E11))*(1+BuyerPremium)+IF(N(Deals!S11)=0,0,MIN(N(Deals!S11),MAX(0,N(Deals!S11)+SheriffCostsFromBid-(N(E11))*(1-RTTPurchase))))),"$#,##0")&amp;" flip profit"))</f>
-        <v/>
+        <v>$138,912 flip profit</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="str">
         <f aca="false">Underwriting!$A12</f>
-        <v/>
+        <v>1311511-9</v>
       </c>
       <c r="B12" s="0" t="str">
         <f aca="false">Underwriting!$B12</f>
-        <v/>
+        <v>9 Gut + $30k foundation, ARV 675k, + $15k estate/title cure</v>
       </c>
       <c r="C12" s="0" t="str">
         <f aca="false">Underwriting!$C12</f>
-        <v/>
-      </c>
-      <c r="D12" s="26" t="str">
+        <v>Flip</v>
+      </c>
+      <c r="D12" s="26" t="n">
         <f aca="false">Underwriting!$D12</f>
-        <v/>
-      </c>
-      <c r="E12" s="8" t="str">
+        <v>137060.071509707</v>
+      </c>
+      <c r="E12" s="8" t="n">
         <f aca="false">IF(Underwriting!$A12="","",Underwriting!$D12)</f>
-        <v/>
+        <v>137060.071509707</v>
       </c>
       <c r="F12" s="11" t="str">
         <f aca="false">IF(Underwriting!$A12="","",IF(Underwriting!$D12&gt;0,"Y","N"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="26" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",N(E12)*(DownPct+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="H12" s="26" t="str">
+        <v>15761.9082236163</v>
+      </c>
+      <c r="H12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IF(N(E12)&gt;0,N(E12)*(1-DownPct)+35,0))</f>
-        <v/>
-      </c>
-      <c r="I12" s="26" t="str">
+        <v>123389.064358737</v>
+      </c>
+      <c r="I12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",IF(C12="Value-add hold",Underwriting!$AA12,Underwriting!$S12)+((N(E12))*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N(E12))*(1-RTTPurchase)))))-N(E12)*(1+BuyerPremium))</f>
-        <v/>
-      </c>
-      <c r="J12" s="26" t="str">
+        <v>341118.7333</v>
+      </c>
+      <c r="J12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",G12+H12+I12)</f>
-        <v/>
-      </c>
-      <c r="K12" s="26" t="str">
+        <v>480269.705882353</v>
+      </c>
+      <c r="K12" s="26" t="n">
         <f aca="false">IF(Underwriting!$A12="","",SUMIF($F$3:F12,"Y",$J$3:J12))</f>
-        <v/>
+        <v>4337842.32700987</v>
       </c>
       <c r="L12" s="0" t="str">
         <f aca="false">IF(Underwriting!$A12="","",IF(C12="Value-add hold",TEXT(IFERROR(Underwriting!$Z12/(((N(E12))*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N(E12))*(1-RTTPurchase)))))+Underwriting!$AA12),0),"0.0%")&amp;" yield on cost",TEXT(Underwriting!$T12-((N(E12))*(1+BuyerPremium)+IF(N(Deals!S12)=0,0,MIN(N(Deals!S12),MAX(0,N(Deals!S12)+SheriffCostsFromBid-(N(E12))*(1-RTTPurchase))))),"$#,##0")&amp;" flip profit"))</f>
-        <v/>
+        <v>$132,065 flip profit</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18828,16 +19004,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B44" s="26" t="n">
         <f aca="false">MAX(0,SUMIF(F3:F42,"Y",G3:G42)-BidderDeposit)</f>
-        <v>144554.252465766</v>
+        <v>212700.407527719</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B45" s="26" t="n">
         <f aca="false">BidderDeposit</f>
@@ -18846,34 +19022,34 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B46" s="26" t="n">
         <f aca="false">SUMIF(F3:F42,"Y",H3:H42)</f>
-        <v>1170599.58451469</v>
+        <v>1704057.31978215</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B47" s="26" t="n">
         <f aca="false">SUMIF(F3:F42,"Y",I3:I42)</f>
-        <v>1096609.6665</v>
+        <v>2416084.5997</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="B48" s="26" t="n">
         <f aca="false">SUMIF(F3:F42,"Y",J3:J42)</f>
-        <v>2416763.50348046</v>
+        <v>4337842.32700987</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B49" s="26" t="n">
         <f aca="false">CapitalCap</f>
@@ -18882,11 +19058,11 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="18" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="B50" s="26" t="n">
         <f aca="false">B49-B48</f>
-        <v>-1416763.50348046</v>
+        <v>-3337842.32700987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>